<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_regionales_migracion)
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_migracion/plot_migracion_miginterna_2019_antofagasta_provincial.xlsx
+++ b/output/graficos_regionales_migracion/plot_migracion_miginterna_2019_antofagasta_provincial.xlsx
@@ -49,7 +49,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-29 18:35</t>
+    <t xml:space="preserve">2026-10-05 04:01</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -504,7 +504,7 @@
         <v>-2.18</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>32.85</v>
+        <v>32.86</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>35.04</v>

</xml_diff>